<commit_message>
Claude Skills have been updated.
</commit_message>
<xml_diff>
--- a/data/sample_data.xlsx
+++ b/data/sample_data.xlsx
@@ -2,14 +2,15 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
+  <workbookProtection/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
-  <calcPr calcId="171027" fullCalcOnLoad="1"/>
+  <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
@@ -25,23 +26,15 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <name val="Calibri"/>
-      <family val="2"/>
       <b val="1"/>
-      <color theme="1"/>
-      <sz val="11"/>
-      <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="2">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
-    </fill>
-    <fill>
-      <patternFill/>
     </fill>
   </fills>
   <borders count="2">
@@ -57,22 +50,21 @@
       <right style="thin"/>
       <top style="thin"/>
       <bottom style="thin"/>
-      <diagonal/>
     </border>
   </borders>
   <cellStyleXfs count="1">
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
   </cellStyles>
-  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
     <indexedColors>
       <rgbColor rgb="00000000"/>
@@ -433,8 +425,8 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P4"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelRow="0"/>
+  <dimension ref="A1:Q4"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
@@ -514,6 +506,11 @@
       </c>
       <c r="P1" s="1" t="inlineStr">
         <is>
+          <t>progress</t>
+        </is>
+      </c>
+      <c r="Q1" s="1" t="inlineStr">
+        <is>
           <t>output_filename</t>
         </is>
       </c>
@@ -596,6 +593,11 @@
       </c>
       <c r="P2" t="inlineStr">
         <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="Q2" t="inlineStr">
+        <is>
           <t>InvitationLetter_Yanai_v2</t>
         </is>
       </c>
@@ -678,6 +680,11 @@
       </c>
       <c r="P3" t="inlineStr">
         <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="Q3" t="inlineStr">
+        <is>
           <t>InvitationLetter_Suzuki_v2</t>
         </is>
       </c>
@@ -760,11 +767,16 @@
       </c>
       <c r="P4" t="inlineStr">
         <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="Q4" t="inlineStr">
+        <is>
           <t>InvitationLetter_Kawashima</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>